<commit_message>
Updated files: BFPat, CCaMC, BIFUbC, BNVP, and TTS
</commit_message>
<xml_diff>
--- a/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
+++ b/InputData/elec/MPCbS/Max Potential Capacity by Source.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/MPCbS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC11F070-45E2-CB41-BBFF-686B3D5B43A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DE5C60-3A8F-2748-B281-7CB583C982AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
     <sheet name="Data-Renewables" sheetId="4" r:id="rId3"/>
-    <sheet name="MPCbS" sheetId="3" r:id="rId4"/>
+    <sheet name="Indonesia Data" sheetId="5" r:id="rId4"/>
+    <sheet name="MPCbS" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="68">
   <si>
     <t>MPCbS Max Potential Capacity by Source</t>
   </si>
@@ -198,6 +199,51 @@
   </si>
   <si>
     <t>https://iesr.or.id/en/pustaka/beyond-207-gigawatts-unleashing-indonesias-solar-potential/#:~:text=A%20geospatial%20assessment%20of%20Indonesia's,land%2Duse%20exclusions%20scenarios).</t>
+  </si>
+  <si>
+    <t>MPCS</t>
+  </si>
+  <si>
+    <t>1 mtoe to MWh</t>
+  </si>
+  <si>
+    <t>1 MWh to MW</t>
+  </si>
+  <si>
+    <t>Biomass (MW)</t>
+  </si>
+  <si>
+    <t>Biomass (mtoe)</t>
+  </si>
+  <si>
+    <t>over a year</t>
+  </si>
+  <si>
+    <t>https://www.eria.org/uploads/media/Research-Project-Report/2022-01-Biomass-Demand-Potential-Indonesia/Forecast-of-Biomass-Demand-Potential-in-Indonesia.pdf</t>
+  </si>
+  <si>
+    <t>https://www.reccessary.com/en/news/Indonesia-wind-power-capacity-target#:~:text=Dewi%20noted%20that%20Indonesia%20has,%2C%20accounting%20for%20about%2040%25.</t>
+  </si>
+  <si>
+    <t>https://www.mdpi.com/2071-1050/17/3/1312</t>
+  </si>
+  <si>
+    <t>https://www.energytransitionpartnership.org/wp-content/uploads/2024/09/20240919-Roadmap-Onshore-Wind-Energy-v5.0-EN.pdf</t>
+  </si>
+  <si>
+    <t>Wind (MW) (total)</t>
+  </si>
+  <si>
+    <t>https://www.reccessary.com/en/news/Indonesia-wind-power-capacity-target</t>
+  </si>
+  <si>
+    <t>Onshore wind (MW)</t>
+  </si>
+  <si>
+    <t>Offshore wind (MW)</t>
+  </si>
+  <si>
+    <t>Geothermal (MW)</t>
   </si>
 </sst>
 </file>
@@ -296,7 +342,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -318,6 +364,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3057,10 +3106,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27209D21-DE46-9B49-910B-40254B76F16A}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>37</v>
       </c>
@@ -3071,7 +3120,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>
@@ -3083,7 +3132,7 @@
         <v>95000</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -3095,7 +3144,7 @@
         <v>60600</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -3106,8 +3155,9 @@
         <f t="shared" si="0"/>
         <v>19835000</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D4" s="10"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
@@ -3120,7 +3170,7 @@
         <v>19835000</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
@@ -3132,7 +3182,7 @@
         <v>32600</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
@@ -3144,7 +3194,7 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -3156,7 +3206,7 @@
         <v>94200</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>35</v>
       </c>
@@ -3168,7 +3218,7 @@
         <v>32600</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>43</v>
       </c>
@@ -3182,6 +3232,129 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66ECDAB1-4503-714B-93D7-817264E3A5A9}">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1"/>
+      <c r="B1" s="15" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3">
+        <v>11630000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4">
+        <f>8760</f>
+        <v>8760</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5">
+        <f>B3/B4</f>
+        <v>1327.6255707762557</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" s="9">
+        <f>B2*B5</f>
+        <v>50449.77168949772</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="9">
+        <v>154600</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15">
+        <v>60400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16">
+        <v>94200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A7" r:id="rId1" xr:uid="{93226CF1-EBC5-E042-BD1F-9F78EF29E2E7}"/>
+    <hyperlink ref="A11" r:id="rId2" location=":~:text=Dewi%20noted%20that%20Indonesia%20has,%2C%20accounting%20for%20about%2040%25." xr:uid="{7779A2B9-5497-404D-91A9-E3D5574598A4}"/>
+    <hyperlink ref="A12" r:id="rId3" xr:uid="{A74447EC-2457-6C4C-9888-8F33B56CEAE2}"/>
+    <hyperlink ref="A13" r:id="rId4" xr:uid="{DDF1EF41-E7EF-5A49-A70F-445F7DA18A1C}"/>
+    <hyperlink ref="A17" r:id="rId5" xr:uid="{1EE2E04A-034A-F64B-AE31-78F1EFAF35E2}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF1F497D"/>
@@ -3277,8 +3450,8 @@
         <v>18</v>
       </c>
       <c r="B9" s="9">
-        <f>'Data-Renewables'!C6</f>
-        <v>32600</v>
+        <f>'Indonesia Data'!B6</f>
+        <v>50449.77168949772</v>
       </c>
       <c r="C9" s="9"/>
     </row>
@@ -3362,7 +3535,9 @@
       </c>
       <c r="C17" s="9"/>
     </row>
-    <row r="21" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="21" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="9"/>
+    </row>
     <row r="22" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="24" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>